<commit_message>
curriculum: add audited master map v0.2
</commit_message>
<xml_diff>
--- a/curriculum/master-map/Mathematics_Understood_Master_Curriculum_Map_v0.2.xlsx
+++ b/curriculum/master-map/Mathematics_Understood_Master_Curriculum_Map_v0.2.xlsx
@@ -1462,7 +1462,7 @@
       </c>
       <c r="C14" s="30" t="inlineStr">
         <is>
-          <t>Representation notes belong in the representation column, not the prerequisite-ID column.</t>
+          <t>Cell-level check confirms representation notes are in the representation column and the prerequisite-ID field is empty.</t>
         </is>
       </c>
     </row>
@@ -1564,22 +1564,22 @@
       </c>
       <c r="D21" s="76" t="inlineStr">
         <is>
-          <t>FND-001 representation notes were placed in Core prerequisite IDs.</t>
+          <t>FND-001 field placement was inspected against the source; representation notes are already in the correct column.</t>
         </is>
       </c>
       <c r="E21" s="76" t="inlineStr">
         <is>
-          <t>Move those notes to Representations / visual requirements and keep prerequisites empty unless actual concept IDs are required.</t>
+          <t>Preserve the correct source data and keep a regression check that the prerequisite column contains concept IDs only.</t>
         </is>
       </c>
       <c r="F21" s="78" t="inlineStr">
         <is>
-          <t>Resolved in v0.2</t>
+          <t>Resolved — verified</t>
         </is>
       </c>
       <c r="G21" s="76" t="inlineStr">
         <is>
-          <t>FND-001 prerequisite cell is empty; representation cell has the notes; prerequisite pairs reconcile.</t>
+          <t>Cell-level check confirms the prerequisite cell is empty and the representation column contains the notes.</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>Audited successor to v0.1. One FND-001 field-alignment issue was corrected. Concepts and dependency interpretations remain provisional pending pedagogical review.</t>
+          <t>Audited successor to v0.1. FND-001 field placement was checked against the source and is already correct. Concepts and dependency interpretations remain provisional pending pedagogical review.</t>
         </is>
       </c>
       <c r="B2" s="1" t="n"/>

</xml_diff>